<commit_message>
Mise à jour pour respect des bonnes pratiques (#139)
* update

* update

* Correction qualité FSH : extensions, exemples et aliases

- MesOriginalData.fsh : correction du ^short copié-collé ("Nombre de jours" → "Valeur originale de la donnée")
- aliases.fsh : centralisation des aliases $loinc, $observation-category, $ContinuaDeviceIdentifiers
- ObservationHb1AcExample.fsh : suppression de la méthode référençant un ValueSet comme CodeSystem
- Renommage des fichiers d'exemples selon la convention *Example.fsh
- sushi-config.yaml : correction du libellé de juridiction ("France" → "France (la)")

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>

---------

Co-authored-by: Claude Sonnet 4.6 <noreply@anthropic.com> 3e75fc24867dc850f818c7e0a872322ea926d5c0
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-mesures-observation-cholesterol-aspect.xlsx
+++ b/main/ig/StructureDefinition-mesures-observation-cholesterol-aspect.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-05-07T07:24:38+00:00</t>
+    <t>2026-06-09T08:46:34+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -646,6 +646,10 @@
     <t>Autres ressources pertinentes *du dossier patient*</t>
   </si>
   <si>
+    <t xml:space="preserve">ele-1
+</t>
+  </si>
+  <si>
     <t>Observation.extension:MesReasonForMeasurement</t>
   </si>
   <si>
@@ -661,10 +665,6 @@
   <si>
     <t>Motif de la mesure
 Texte libre (ex. diabète, surpoids, hypercholestérolémie, risque cardiovasculaire, suivi, ...)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ele-1
-</t>
   </si>
   <si>
     <t>Observation.extension:mes-original-data</t>
@@ -4281,7 +4281,7 @@
         <v>81</v>
       </c>
       <c r="AI18" t="s" s="2">
-        <v>82</v>
+        <v>202</v>
       </c>
       <c r="AJ18" t="s" s="2">
         <v>122</v>
@@ -4307,13 +4307,13 @@
     </row>
     <row r="19" hidden="true">
       <c r="A19" t="s" s="2">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B19" t="s" s="2">
         <v>193</v>
       </c>
       <c r="C19" t="s" s="2">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="D19" t="s" s="2">
         <v>82</v>
@@ -4335,13 +4335,13 @@
         <v>82</v>
       </c>
       <c r="K19" t="s" s="2">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="L19" t="s" s="2">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="M19" t="s" s="2">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="N19" s="2"/>
       <c r="O19" s="2"/>
@@ -4401,7 +4401,7 @@
         <v>81</v>
       </c>
       <c r="AI19" t="s" s="2">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="AJ19" t="s" s="2">
         <v>122</v>
@@ -4521,7 +4521,7 @@
         <v>81</v>
       </c>
       <c r="AI20" t="s" s="2">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="AJ20" t="s" s="2">
         <v>122</v>

</xml_diff>